<commit_message>
feat(eval): integrar evaluacion dual con TypeSafe AI Jev (System One) y Gemini 3.5 Flash Judge
</commit_message>
<xml_diff>
--- a/data/results/banco_pruebas_50.xlsx
+++ b/data/results/banco_pruebas_50.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Normativa y Trámites</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Normativa y Trámites</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Normativa y Trámites</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Normativa y Trámites</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Normativa y Trámites</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Matrícula y Registros</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Biblioteca Virtual</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Campus Virtual y Aprendizaje</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Normativa y Trámites</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Matrícula y Registros Académicos</t>
+          <t>Pagos y Cobranzas</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">

</xml_diff>